<commit_message>
datos: +0 Kino, +1 Pool hasta 2026-09-25
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B250"/>
+  <dimension ref="A1:B251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12038,6 +12038,18 @@
       <c r="B250" s="2" t="inlineStr">
         <is>
           <t>12, 20, 21, 24, 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25  Vie</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>01, 04, 18, 26, 31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +0 Kino, +1 Pool hasta 2026-10-03
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B258"/>
+  <dimension ref="A1:B259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12134,6 +12134,18 @@
       <c r="B258" s="2" t="inlineStr">
         <is>
           <t>04, 05, 06, 27, 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03  Sáb</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>03, 15, 21, 25, 30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +0 Kino, +1 Pool hasta 2026-10-10
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B265"/>
+  <dimension ref="A1:B266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12218,6 +12218,18 @@
       <c r="B265" s="2" t="inlineStr">
         <is>
           <t>08, 10, 15, 18, 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10  Sáb</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>03, 05, 13, 18, 30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +0 Kino, +1 Pool hasta 2026-10-11
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B266"/>
+  <dimension ref="A1:B267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12230,6 +12230,18 @@
       <c r="B266" s="2" t="inlineStr">
         <is>
           <t>03, 05, 13, 18, 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11  Dom</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>11, 13, 15, 18, 26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-18
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B273"/>
+  <dimension ref="A1:B274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12314,6 +12314,18 @@
       <c r="B273" s="2" t="inlineStr">
         <is>
           <t>02, 13, 15, 20, 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18  Dom</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>02, 11, 15, 26, 28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-19
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B274"/>
+  <dimension ref="A1:B275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12326,6 +12326,18 @@
       <c r="B274" s="2" t="inlineStr">
         <is>
           <t>02, 11, 15, 26, 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19  Lun</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>03, 18, 28, 29, 31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-20
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B275"/>
+  <dimension ref="A1:B276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12338,6 +12338,18 @@
       <c r="B275" s="2" t="inlineStr">
         <is>
           <t>03, 18, 28, 29, 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20  Mar</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>16, 18, 19, 20, 30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-21
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B276"/>
+  <dimension ref="A1:B277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12350,6 +12350,18 @@
       <c r="B276" s="2" t="inlineStr">
         <is>
           <t>16, 18, 19, 20, 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21  Mié</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>12, 16, 24, 30, 31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-22
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B277"/>
+  <dimension ref="A1:B278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12362,6 +12362,18 @@
       <c r="B277" s="2" t="inlineStr">
         <is>
           <t>12, 16, 24, 30, 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22  Jue</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>02, 08, 09, 21, 23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-23
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B278"/>
+  <dimension ref="A1:B279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12374,6 +12374,18 @@
       <c r="B278" s="2" t="inlineStr">
         <is>
           <t>02, 08, 09, 21, 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23  Vie</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>14, 16, 19, 28, 31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-24
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B279"/>
+  <dimension ref="A1:B280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12386,6 +12386,18 @@
       <c r="B279" s="2" t="inlineStr">
         <is>
           <t>14, 16, 19, 28, 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24  Sáb</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>10, 12, 14, 21, 24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-25
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B280"/>
+  <dimension ref="A1:B281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12398,6 +12398,18 @@
       <c r="B280" s="2" t="inlineStr">
         <is>
           <t>10, 12, 14, 21, 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25  Dom</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>03, 09, 16, 27, 29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-26
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B281"/>
+  <dimension ref="A1:B282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12410,6 +12410,18 @@
       <c r="B281" s="2" t="inlineStr">
         <is>
           <t>03, 09, 16, 27, 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26  Lun</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>21, 22, 23, 26, 28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +0 Kino, +1 Pool hasta 2026-10-27
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B282"/>
+  <dimension ref="A1:B283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12422,6 +12422,18 @@
       <c r="B282" s="2" t="inlineStr">
         <is>
           <t>21, 22, 23, 26, 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27  Mar</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>03, 11, 16, 18, 20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +0 Kino, +1 Pool hasta 2026-10-28
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B283"/>
+  <dimension ref="A1:B284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12434,6 +12434,18 @@
       <c r="B283" s="2" t="inlineStr">
         <is>
           <t>03, 11, 16, 18, 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28  Mié</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>01, 13, 15, 20, 28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-29
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -9043,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B284"/>
+  <dimension ref="A1:B285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12446,6 +12446,18 @@
       <c r="B284" s="2" t="inlineStr">
         <is>
           <t>01, 13, 15, 20, 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29  Jue</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>02, 04, 11, 26, 29</t>
         </is>
       </c>
     </row>

</xml_diff>